<commit_message>
AI 投資地圖 v0.6.17 重抽：併入 main 上的 Amazon v0.3.1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V11Bcxj2uwkRVE7mK2RCtH
</commit_message>
<xml_diff>
--- a/markets/invest_map/dist/20261031_AI投資地圖_資料_v0.6.17.xlsx
+++ b/markets/invest_map/dist/20261031_AI投資地圖_資料_v0.6.17.xlsx
@@ -6283,16 +6283,16 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>249.09</v>
+        <v>240.35</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>amazon/dist/20261027_Amazon個股模型_v0.3.xlsx Val!B20</t>
+          <t>amazon/dist/20261031_Amazon個股模型_v0.3.1.xlsx Val!B20</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
@@ -9928,19 +9928,19 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>215.578882385843</v>
+        <v>217.650781868569</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>amazon/dist/20261027_Amazon個股模型_v0.3.xlsx Val!B19</t>
+          <t>amazon/dist/20261031_Amazon個股模型_v0.3.1.xlsx Val!B19</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>117.352344636521</v>
+        <v>120.190250466792</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>amazon/dist/20261027_Amazon個股模型_v0.3.xlsx Val!D5</t>
+          <t>amazon/dist/20261031_Amazon個股模型_v0.3.1.xlsx Val!D5</t>
         </is>
       </c>
       <c r="N16">
@@ -9956,7 +9956,7 @@
         <v/>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>-0.134534174853092</v>
+        <v>-0.09444234712474051</v>
       </c>
       <c r="R16">
         <f>P16/N16-1</f>
@@ -9969,7 +9969,7 @@
       </c>
       <c r="W16" s="1" t="inlineStr">
         <is>
-          <t>DCF 目標價 149.6（Val!B17）；Comparable 目標價 281.6（Val!B18）；市場共識目標價 332.2（Val!B25，外部、僅供對照）；價格帶 C～A 情境 DCF 117.4～205.0</t>
+          <t>DCF 目標價 147.3（Val!B17）；Comparable 目標價 288.0（Val!B18）；市場共識目標價 332.4（Val!B25，外部、僅供對照）；價格帶 C～A 情境 DCF 120.2～193.2</t>
         </is>
       </c>
       <c r="Z16">
@@ -9987,23 +9987,23 @@
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>自由現金流扣股利五年合計（基準情境 B；A 205.5、C -43.2）</t>
+          <t>自由現金流扣股利五年合計（基準情境 B；A 258.3、C 37.7）</t>
         </is>
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>情境 B 五年合計 19.0</t>
+          <t>情境 B 五年合計 89.6</t>
         </is>
       </c>
       <c r="AE16" s="4" t="n">
-        <v>19.0072988716234</v>
+        <v>89.6117652783997</v>
       </c>
       <c r="AF16" s="4" t="n">
-        <v>19.0072988716234</v>
+        <v>89.6117652783997</v>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>[Derived] amazon/dist/20261027_Amazon個股模型_v0.3.xlsx CF!C6…CF!C6</t>
+          <t>[Derived] amazon/dist/20261031_Amazon個股模型_v0.3.1.xlsx CF!C6…CF!C6</t>
         </is>
       </c>
       <c r="AH16">
@@ -10021,7 +10021,7 @@
       </c>
       <c r="AK16" s="1" t="inlineStr">
         <is>
-          <t>上檔空間 amazon/dist/20261027_Amazon個股模型_v0.3.xlsx Val!B21；投資建議 amazon/dist/20261027_Amazon個股模型_v0.3.xlsx Val!B24；級距 amazon/dist/20261027_Amazon個股模型_v0.3.xlsx Val!B23</t>
+          <t>上檔空間 amazon/dist/20261031_Amazon個股模型_v0.3.1.xlsx Val!B21；投資建議 amazon/dist/20261031_Amazon個股模型_v0.3.1.xlsx Val!B24；級距 amazon/dist/20261031_Amazon個股模型_v0.3.1.xlsx Val!B23</t>
         </is>
       </c>
     </row>
@@ -11257,14 +11257,14 @@
         </is>
       </c>
       <c r="AE27" s="4" t="n">
-        <v>107.6782012460332</v>
+        <v>107.5108808028628</v>
       </c>
       <c r="AF27" s="4" t="n">
-        <v>-18.5037194506051</v>
+        <v>-18.5249393183946</v>
       </c>
       <c r="AG27" t="inlineStr">
         <is>
-          <t>[Derived] anthropic/dist/20261024_Anthropic收支模型_v0_1_5.xlsx Funding!E14…Funding!I14</t>
+          <t>[Derived] anthropic/dist/20261031_Anthropic收支模型_v0_1_6.xlsx Funding!E14…Funding!I14</t>
         </is>
       </c>
       <c r="AH27">

</xml_diff>